<commit_message>
feat: add some files in 'frequencias' folder
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9396AF1A-4CA9-490D-B2D6-BF2F9E48B3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9575FDC-42D2-47C6-A44E-5EAFC0688D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>APENADO</t>
   </si>
@@ -94,19 +94,28 @@
   </si>
   <si>
     <t>ROBERTO WILSON MOURA FILHO(MAXSUEL)</t>
+  </si>
+  <si>
+    <t>PAULO RICARDO CANUTO GUEDES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -162,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -171,18 +180,28 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EF9E8C-546D-4B9E-9D3D-4B096DC9D66B}">
-  <dimension ref="D9:J19"/>
+  <dimension ref="D9:J21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="17.21875" customWidth="1"/>
@@ -511,15 +530,15 @@
   </cols>
   <sheetData>
     <row r="9" spans="4:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9" t="s">
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="9"/>
+      <c r="H9" s="6"/>
       <c r="I9" s="2" t="s">
         <v>4</v>
       </c>
@@ -528,15 +547,15 @@
       </c>
     </row>
     <row r="10" spans="4:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="8" t="s">
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H10" s="8"/>
+      <c r="H10" s="7"/>
       <c r="I10" s="3">
         <v>45870</v>
       </c>
@@ -545,15 +564,15 @@
       </c>
     </row>
     <row r="11" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="7" t="s">
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="8"/>
       <c r="I11" s="3">
         <v>45778</v>
       </c>
@@ -562,15 +581,15 @@
       </c>
     </row>
     <row r="12" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="7" t="s">
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="8"/>
       <c r="I12" s="3">
         <v>45778</v>
       </c>
@@ -579,15 +598,15 @@
       </c>
     </row>
     <row r="13" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="7" t="s">
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="8"/>
       <c r="I13" s="3">
         <v>45901</v>
       </c>
@@ -596,15 +615,15 @@
       </c>
     </row>
     <row r="14" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="7" t="s">
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="8"/>
       <c r="I14" s="3">
         <v>45778</v>
       </c>
@@ -613,15 +632,15 @@
       </c>
     </row>
     <row r="15" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="7" t="s">
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="8"/>
       <c r="I15" s="3">
         <v>45992</v>
       </c>
@@ -630,15 +649,15 @@
       </c>
     </row>
     <row r="16" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="7" t="s">
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="8"/>
       <c r="I16" s="3">
         <v>45992</v>
       </c>
@@ -647,50 +666,62 @@
       </c>
     </row>
     <row r="17" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
+      <c r="J17" s="3"/>
     </row>
     <row r="18" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
+      <c r="J18" s="3"/>
     </row>
     <row r="19" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="D20" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="9"/>
+      <c r="I20" s="12">
+        <v>46113</v>
+      </c>
+      <c r="J20" s="3">
+        <v>46478</v>
+      </c>
+    </row>
+    <row r="21" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="J21" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
+  <mergeCells count="24">
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:H20"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="D18:F18"/>
@@ -703,7 +734,18 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update 'apostilamento-frequencias' in 'frequencias' folder
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9575FDC-42D2-47C6-A44E-5EAFC0688D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DD610D-B116-4C6C-9A31-7642E332A3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
@@ -180,14 +180,12 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -195,13 +193,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,15 +530,15 @@
   </cols>
   <sheetData>
     <row r="9" spans="4:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6" t="s">
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="6"/>
+      <c r="H9" s="13"/>
       <c r="I9" s="2" t="s">
         <v>4</v>
       </c>
@@ -552,15 +552,15 @@
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="12"/>
       <c r="I10" s="3">
         <v>45870</v>
       </c>
       <c r="J10" s="5">
-        <v>46082</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="4:10" x14ac:dyDescent="0.3">
@@ -569,10 +569,10 @@
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="8"/>
+      <c r="H11" s="11"/>
       <c r="I11" s="3">
         <v>45778</v>
       </c>
@@ -586,10 +586,10 @@
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="8"/>
+      <c r="H12" s="11"/>
       <c r="I12" s="3">
         <v>45778</v>
       </c>
@@ -603,10 +603,10 @@
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="8"/>
+      <c r="H13" s="11"/>
       <c r="I13" s="3">
         <v>45901</v>
       </c>
@@ -620,10 +620,10 @@
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="8"/>
+      <c r="H14" s="11"/>
       <c r="I14" s="3">
         <v>45778</v>
       </c>
@@ -637,10 +637,10 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="8"/>
+      <c r="H15" s="11"/>
       <c r="I15" s="3">
         <v>45992</v>
       </c>
@@ -654,10 +654,10 @@
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="8"/>
+      <c r="H16" s="11"/>
       <c r="I16" s="3">
         <v>45992</v>
       </c>
@@ -671,8 +671,8 @@
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
       <c r="I17" s="1"/>
       <c r="J17" s="3"/>
     </row>
@@ -682,10 +682,12 @@
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="3"/>
+      <c r="J18" s="4">
+        <v>46082</v>
+      </c>
     </row>
     <row r="19" spans="4:10" x14ac:dyDescent="0.3">
       <c r="D19" s="10" t="s">
@@ -693,22 +695,22 @@
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
       <c r="I19" s="1"/>
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
       <c r="G20" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H20" s="9"/>
-      <c r="I20" s="12">
+      <c r="I20" s="6">
         <v>46113</v>
       </c>
       <c r="J20" s="3">
@@ -716,10 +718,20 @@
       </c>
     </row>
     <row r="21" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="J21" s="13"/>
+      <c r="J21" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="D14:F14"/>
@@ -734,16 +746,6 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: update 'apostilamento-frequencias' in 'frequancias' folders at 27/04/2026
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DD610D-B116-4C6C-9A31-7642E332A3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A9937A1-FC57-41DA-BB53-90E3760AE1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>APENADO</t>
   </si>
@@ -97,13 +97,22 @@
   </si>
   <si>
     <t>PAULO RICARDO CANUTO GUEDES</t>
+  </si>
+  <si>
+    <t>JOSIMAR FREIRE DA SILVA</t>
+  </si>
+  <si>
+    <t>5 MESES</t>
+  </si>
+  <si>
+    <t>2 ANOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,6 +125,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -171,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -183,23 +198,22 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -516,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EF9E8C-546D-4B9E-9D3D-4B096DC9D66B}">
-  <dimension ref="D9:J21"/>
+  <dimension ref="D9:J22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="17.21875" customWidth="1"/>
@@ -530,15 +544,15 @@
   </cols>
   <sheetData>
     <row r="9" spans="4:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13" t="s">
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="13"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="2" t="s">
         <v>4</v>
       </c>
@@ -547,15 +561,15 @@
       </c>
     </row>
     <row r="10" spans="4:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="12" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="H10" s="12"/>
+      <c r="H10" s="9"/>
       <c r="I10" s="3">
         <v>45870</v>
       </c>
@@ -564,15 +578,15 @@
       </c>
     </row>
     <row r="11" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="11" t="s">
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="10"/>
       <c r="I11" s="3">
         <v>45778</v>
       </c>
@@ -581,15 +595,15 @@
       </c>
     </row>
     <row r="12" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="11" t="s">
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="11"/>
+      <c r="H12" s="10"/>
       <c r="I12" s="3">
         <v>45778</v>
       </c>
@@ -598,15 +612,15 @@
       </c>
     </row>
     <row r="13" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="11" t="s">
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="10"/>
       <c r="I13" s="3">
         <v>45901</v>
       </c>
@@ -615,15 +629,15 @@
       </c>
     </row>
     <row r="14" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="11" t="s">
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="11"/>
+      <c r="H14" s="10"/>
       <c r="I14" s="3">
         <v>45778</v>
       </c>
@@ -632,15 +646,15 @@
       </c>
     </row>
     <row r="15" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="11" t="s">
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="11"/>
+      <c r="H15" s="10"/>
       <c r="I15" s="3">
         <v>45992</v>
       </c>
@@ -649,15 +663,15 @@
       </c>
     </row>
     <row r="16" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="11" t="s">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="11"/>
+      <c r="H16" s="10"/>
       <c r="I16" s="3">
         <v>45992</v>
       </c>
@@ -666,50 +680,50 @@
       </c>
     </row>
     <row r="17" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
       <c r="I17" s="1"/>
       <c r="J17" s="3"/>
     </row>
     <row r="18" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
       <c r="I18" s="1"/>
       <c r="J18" s="4">
         <v>46082</v>
       </c>
     </row>
     <row r="19" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
       <c r="I19" s="1"/>
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="9" t="s">
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H20" s="9"/>
+      <c r="H20" s="12"/>
       <c r="I20" s="6">
         <v>46113</v>
       </c>
@@ -718,20 +732,45 @@
       </c>
     </row>
     <row r="21" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="J21" s="7"/>
+      <c r="D21" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="12"/>
+      <c r="I21" s="6">
+        <v>46143</v>
+      </c>
+      <c r="J21" s="3">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="22" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="D22" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="12"/>
+      <c r="I22" s="6">
+        <v>46143</v>
+      </c>
+      <c r="J22" s="3">
+        <v>46874</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
+  <mergeCells count="28">
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:H22"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="D14:F14"/>
@@ -746,7 +785,18 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update 'apostilamento-frequencias' files and add 'frequencias-capa' for 04/2026 and 05/2026
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4D4B79-3164-4F0B-8119-5EF15C890B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3B7F61-8201-46A9-B4ED-0AFB9993D5A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
@@ -210,17 +210,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,15 +550,15 @@
   </cols>
   <sheetData>
     <row r="9" spans="4:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12" t="s">
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="12"/>
+      <c r="H9" s="9"/>
       <c r="I9" s="2" t="s">
         <v>4</v>
       </c>
@@ -567,11 +567,11 @@
       </c>
     </row>
     <row r="10" spans="4:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
       <c r="G10" s="11" t="s">
         <v>3</v>
       </c>
@@ -579,37 +579,37 @@
       <c r="I10" s="3">
         <v>45870</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="10" t="s">
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="10"/>
+      <c r="H11" s="12"/>
       <c r="I11" s="3">
         <v>45778</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="4">
         <v>46023</v>
       </c>
     </row>
     <row r="12" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10" t="s">
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="10"/>
+      <c r="H12" s="12"/>
       <c r="I12" s="3">
         <v>45778</v>
       </c>
@@ -618,15 +618,15 @@
       </c>
     </row>
     <row r="13" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="10" t="s">
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="10"/>
+      <c r="H13" s="12"/>
       <c r="I13" s="3">
         <v>45901</v>
       </c>
@@ -635,88 +635,88 @@
       </c>
     </row>
     <row r="14" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="10" t="s">
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="10"/>
+      <c r="H14" s="12"/>
       <c r="I14" s="3">
         <v>45778</v>
       </c>
-      <c r="J14" s="3">
+      <c r="J14" s="5">
         <v>46174</v>
       </c>
     </row>
     <row r="15" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="10" t="s">
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="10"/>
+      <c r="H15" s="12"/>
       <c r="I15" s="3">
         <v>45992</v>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="5">
         <v>46327</v>
       </c>
     </row>
     <row r="16" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="10" t="s">
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="10"/>
+      <c r="H16" s="12"/>
       <c r="I16" s="3">
         <v>45992</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="5">
         <v>46327</v>
       </c>
     </row>
     <row r="17" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
       <c r="I17" s="1"/>
       <c r="J17" s="3"/>
     </row>
     <row r="18" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
       <c r="I18" s="1"/>
       <c r="J18" s="4">
         <v>46082</v>
       </c>
     </row>
     <row r="19" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
       <c r="I19" s="1"/>
       <c r="J19" s="3"/>
     </row>
@@ -750,7 +750,7 @@
       <c r="I21" s="6">
         <v>46143</v>
       </c>
-      <c r="J21" s="3">
+      <c r="J21" s="5">
         <v>46266</v>
       </c>
     </row>
@@ -790,6 +790,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="G23:H23"/>
     <mergeCell ref="D9:F9"/>
@@ -806,20 +820,6 @@
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:H20"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
docs: update 'apostilamento-frequencias' in 'frequencias' folder
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3B7F61-8201-46A9-B4ED-0AFB9993D5A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08A45E9-9539-4E0A-9446-05E91958DAB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
   <si>
     <t>APENADO</t>
   </si>
@@ -45,12 +45,6 @@
     <t>JOSIMAR FIALHO DA SILVA</t>
   </si>
   <si>
-    <t>PENA</t>
-  </si>
-  <si>
-    <t>7 MESES E 7 HORAS</t>
-  </si>
-  <si>
     <t>INICIO</t>
   </si>
   <si>
@@ -112,13 +106,46 @@
   </si>
   <si>
     <t>1 ANO E 4 MESES</t>
+  </si>
+  <si>
+    <t>PROCESSO Nº</t>
+  </si>
+  <si>
+    <t>FREQUÊNCIAS</t>
+  </si>
+  <si>
+    <t>9000028-15.2022.8.15.0561</t>
+  </si>
+  <si>
+    <t>PERIODO DA PRESTAÇÃO</t>
+  </si>
+  <si>
+    <t>DATA</t>
+  </si>
+  <si>
+    <t>HORA</t>
+  </si>
+  <si>
+    <t>9000010-86.2025.8.15.0561</t>
+  </si>
+  <si>
+    <t>0800548-27.2024.8.15.0561</t>
+  </si>
+  <si>
+    <t>7 MESES</t>
+  </si>
+  <si>
+    <t>0800141-26.2021.8.15.0561</t>
+  </si>
+  <si>
+    <t>PERIODO EM MESES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,19 +154,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -164,8 +198,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -188,39 +228,103 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,292 +640,421 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EF9E8C-546D-4B9E-9D3D-4B096DC9D66B}">
-  <dimension ref="D9:J23"/>
+  <dimension ref="B8:L23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="17.21875" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" customWidth="1"/>
-    <col min="11" max="11" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="28.21875" customWidth="1"/>
+    <col min="5" max="5" width="17.21875" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" customWidth="1"/>
+    <col min="9" max="9" width="14.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" customWidth="1"/>
+    <col min="12" max="12" width="13.88671875" customWidth="1"/>
+    <col min="13" max="13" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="4:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="9" t="s">
+    <row r="8" spans="2:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="2:12" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9" t="s">
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="2" t="s">
+      <c r="L9" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="18">
+        <v>7</v>
+      </c>
+      <c r="K10" s="9">
+        <v>45870</v>
+      </c>
+      <c r="L10" s="10">
+        <v>46026</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" s="11"/>
+      <c r="J11" s="20">
+        <v>8</v>
+      </c>
+      <c r="K11" s="9">
+        <v>45778</v>
+      </c>
+      <c r="L11" s="10">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="15">
+        <v>45771</v>
+      </c>
+      <c r="C12" s="16">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="4:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D10" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="3">
-        <v>45870</v>
-      </c>
-      <c r="J10" s="4">
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="I12" s="11"/>
+      <c r="J12" s="20">
+        <v>8</v>
+      </c>
+      <c r="K12" s="9">
+        <v>45778</v>
+      </c>
+      <c r="L12" s="10">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="I13" s="11"/>
+      <c r="J13" s="20">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D11" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="12"/>
-      <c r="I11" s="3">
+      <c r="K13" s="9">
+        <v>45901</v>
+      </c>
+      <c r="L13" s="10">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" s="11"/>
+      <c r="J14" s="20">
+        <v>14</v>
+      </c>
+      <c r="K14" s="9">
         <v>45778</v>
       </c>
-      <c r="J11" s="4">
-        <v>46023</v>
-      </c>
-    </row>
-    <row r="12" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D12" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" s="12"/>
-      <c r="I12" s="3">
-        <v>45778</v>
-      </c>
-      <c r="J12" s="4">
+      <c r="L14" s="12">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="11"/>
+      <c r="J15" s="20">
+        <v>12</v>
+      </c>
+      <c r="K15" s="9">
         <v>45992</v>
       </c>
-    </row>
-    <row r="13" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D13" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H13" s="12"/>
-      <c r="I13" s="3">
-        <v>45901</v>
-      </c>
-      <c r="J13" s="4">
+      <c r="L15" s="12">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="11"/>
+      <c r="J16" s="20">
+        <v>12</v>
+      </c>
+      <c r="K16" s="9">
         <v>45992</v>
       </c>
-    </row>
-    <row r="14" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D14" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="12" t="s">
+      <c r="L16" s="12">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="9"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="10">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="9"/>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="12"/>
-      <c r="I14" s="3">
-        <v>45778</v>
-      </c>
-      <c r="J14" s="5">
-        <v>46174</v>
-      </c>
-    </row>
-    <row r="15" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D15" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" s="12"/>
-      <c r="I15" s="3">
-        <v>45992</v>
-      </c>
-      <c r="J15" s="5">
-        <v>46327</v>
-      </c>
-    </row>
-    <row r="16" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D16" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="12"/>
-      <c r="I16" s="3">
-        <v>45992</v>
-      </c>
-      <c r="J16" s="5">
-        <v>46327</v>
-      </c>
-    </row>
-    <row r="17" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D17" s="10" t="s">
+      <c r="I20" s="2"/>
+      <c r="J20" s="21">
+        <v>12</v>
+      </c>
+      <c r="K20" s="14">
+        <v>46113</v>
+      </c>
+      <c r="L20" s="9">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B21" s="15">
+        <v>46094</v>
+      </c>
+      <c r="C21" s="16">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I21" s="2"/>
+      <c r="J21" s="21">
+        <v>5</v>
+      </c>
+      <c r="K21" s="14">
+        <v>46143</v>
+      </c>
+      <c r="L21" s="12">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I22" s="2"/>
+      <c r="J22" s="21">
+        <v>24</v>
+      </c>
+      <c r="K22" s="14">
+        <v>46143</v>
+      </c>
+      <c r="L22" s="9">
+        <v>46844</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B23" s="15">
+        <v>46094</v>
+      </c>
+      <c r="C23" s="16">
+        <v>0.375</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I23" s="2"/>
+      <c r="J23" s="21">
         <v>16</v>
       </c>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="3"/>
-    </row>
-    <row r="18" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D18" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="4">
-        <v>46082</v>
-      </c>
-    </row>
-    <row r="19" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D19" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D20" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="8"/>
-      <c r="I20" s="6">
-        <v>46113</v>
-      </c>
-      <c r="J20" s="3">
-        <v>46447</v>
-      </c>
-    </row>
-    <row r="21" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D21" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="6">
+      <c r="K23" s="14">
         <v>46143</v>
       </c>
-      <c r="J21" s="5">
-        <v>46266</v>
-      </c>
-    </row>
-    <row r="22" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D22" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="6">
-        <v>46143</v>
-      </c>
-      <c r="J22" s="3">
-        <v>46844</v>
-      </c>
-    </row>
-    <row r="23" spans="4:10" x14ac:dyDescent="0.3">
-      <c r="D23" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="6">
-        <v>46143</v>
-      </c>
-      <c r="J23" s="3">
+      <c r="L23" s="9">
         <v>46600</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D19:F19"/>
+  <mergeCells count="31">
+    <mergeCell ref="B8:L8"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E17:G17"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add 'frequencias' referring to 05/2026 and add 'junho' folder in 'frequencias'
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -8,15 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D06A9119-3851-499E-866A-BB71236362C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E1B7DF-FF53-4B39-AB9F-D7CFE9D19546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
   <sheets>
-    <sheet name="Main" sheetId="1" r:id="rId1"/>
+    <sheet name="MAIN" sheetId="1" r:id="rId1"/>
     <sheet name="2025" sheetId="3" r:id="rId2"/>
     <sheet name="2026" sheetId="2" r:id="rId3"/>
+    <sheet name="CONFIG" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="status_list">tbl_status[status_id]</definedName>
+    <definedName name="status_name_list">tbl_status[display_name]</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="96">
   <si>
     <t>APENADO</t>
   </si>
@@ -215,20 +220,125 @@
     <t>DEZEMBRO</t>
   </si>
   <si>
-    <t>!</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>9000034-17.2025.8.15.0561</t>
+  </si>
+  <si>
+    <t>ISMAELY DE LIMA ALVES</t>
+  </si>
+  <si>
+    <t>1  ANO</t>
+  </si>
+  <si>
+    <t>9000002-80.2023.8.15.0561</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>status_id</t>
+  </si>
+  <si>
+    <t>display_name</t>
+  </si>
+  <si>
+    <t>SENT</t>
+  </si>
+  <si>
+    <t>PENDING</t>
+  </si>
+  <si>
+    <t>ENVIADO</t>
+  </si>
+  <si>
+    <t>PENDENTE</t>
+  </si>
+  <si>
+    <t>BLANK</t>
+  </si>
+  <si>
+    <t>IN_PROGRESS</t>
+  </si>
+  <si>
+    <t>NÃO INICIADO</t>
+  </si>
+  <si>
+    <t>NOT_STARTED</t>
+  </si>
+  <si>
+    <t>EM PROGRESSO</t>
+  </si>
+  <si>
+    <t>SUÊNIO GREGÓRIO</t>
+  </si>
+  <si>
+    <t>0801047-74.2025.8.15.0561</t>
+  </si>
+  <si>
+    <t>MANOEL DE LIMA</t>
+  </si>
+  <si>
+    <t>9000039-39.2025.8.15.0561</t>
+  </si>
+  <si>
+    <t>JOSÉ NEUDO GARRIDO DE ANDRADE</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>AF0001</t>
+  </si>
+  <si>
+    <t>AF0002</t>
+  </si>
+  <si>
+    <t>AF0003</t>
+  </si>
+  <si>
+    <t>AF0004</t>
+  </si>
+  <si>
+    <t>AF0005</t>
+  </si>
+  <si>
+    <t>AF0006</t>
+  </si>
+  <si>
+    <t>AF0007</t>
+  </si>
+  <si>
+    <t>AF0008</t>
+  </si>
+  <si>
+    <t>AF0009</t>
+  </si>
+  <si>
+    <t>AF0010</t>
+  </si>
+  <si>
+    <t>AF0011</t>
+  </si>
+  <si>
+    <t>AF0012</t>
+  </si>
+  <si>
+    <t>AF0013</t>
+  </si>
+  <si>
+    <t>AF0014</t>
+  </si>
+  <si>
+    <t>AF0015</t>
+  </si>
+  <si>
+    <t>AF0016</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -255,8 +365,24 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -293,8 +419,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -330,11 +462,90 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -378,6 +589,36 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -395,27 +636,21 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="11">
     <dxf>
       <font>
         <b/>
@@ -423,268 +658,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -717,9 +691,114 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -732,6 +811,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67B21386-A7FE-4230-BF7C-AC6702050BBE}" name="tbl_status" displayName="tbl_status" ref="B3:C8" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+  <autoFilter ref="B3:C8" xr:uid="{67B21386-A7FE-4230-BF7C-AC6702050BBE}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{8CA856E5-CBA8-4981-BAC5-458B8D165D4E}" name="status_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{DEF6E58C-573F-4688-813D-EB15040558D7}" name="display_name" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1031,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EF9E8C-546D-4B9E-9D3D-4B096DC9D66B}">
-  <dimension ref="A1:R37"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="28.21875" customWidth="1"/>
@@ -1189,17 +1282,17 @@
     <row r="8" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
@@ -1214,15 +1307,15 @@
       <c r="C9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="22" t="s">
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="22"/>
+      <c r="H9" s="36"/>
       <c r="I9" s="8" t="s">
         <v>30</v>
       </c>
@@ -1246,15 +1339,15 @@
       <c r="C10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17" t="s">
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="17"/>
+      <c r="H10" s="31"/>
       <c r="I10" s="7">
         <v>7</v>
       </c>
@@ -1278,15 +1371,15 @@
       <c r="C11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="18" t="s">
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="H11" s="18"/>
+      <c r="H11" s="32"/>
       <c r="I11" s="9">
         <v>8</v>
       </c>
@@ -1310,15 +1403,15 @@
       <c r="C12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="18" t="s">
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="18"/>
+      <c r="H12" s="32"/>
       <c r="I12" s="9">
         <v>8</v>
       </c>
@@ -1342,15 +1435,15 @@
       <c r="C13" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="18" t="s">
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="18"/>
+      <c r="H13" s="32"/>
       <c r="I13" s="9">
         <v>4</v>
       </c>
@@ -1374,15 +1467,15 @@
       <c r="C14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18" t="s">
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="18"/>
+      <c r="H14" s="32"/>
       <c r="I14" s="9">
         <v>14</v>
       </c>
@@ -1406,15 +1499,15 @@
       <c r="C15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="18" t="s">
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="18"/>
+      <c r="H15" s="32"/>
       <c r="I15" s="9">
         <v>12</v>
       </c>
@@ -1438,15 +1531,15 @@
       <c r="C16" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="18" t="s">
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="H16" s="18"/>
+      <c r="H16" s="32"/>
       <c r="I16" s="9">
         <v>12</v>
       </c>
@@ -1470,15 +1563,15 @@
       <c r="C17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H17" s="18"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" s="32"/>
       <c r="I17" s="9" t="s">
         <v>31</v>
       </c>
@@ -1498,15 +1591,15 @@
       <c r="C18" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="18"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H18" s="32"/>
       <c r="I18" s="9" t="s">
         <v>31</v>
       </c>
@@ -1528,15 +1621,15 @@
       <c r="C19" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" s="18"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" s="32"/>
       <c r="I19" s="9" t="s">
         <v>31</v>
       </c>
@@ -1554,15 +1647,15 @@
       <c r="A20" s="16"/>
       <c r="B20" s="16"/>
       <c r="C20" s="7"/>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19" t="s">
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="19"/>
+      <c r="H20" s="33"/>
       <c r="I20" s="10">
         <v>12</v>
       </c>
@@ -1586,15 +1679,15 @@
       <c r="C21" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19" t="s">
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="H21" s="19"/>
+      <c r="H21" s="33"/>
       <c r="I21" s="10">
         <v>5</v>
       </c>
@@ -1618,15 +1711,15 @@
       <c r="C22" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19" t="s">
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="H22" s="19"/>
+      <c r="H22" s="33"/>
       <c r="I22" s="10">
         <v>24</v>
       </c>
@@ -1650,23 +1743,23 @@
       <c r="C23" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19" t="s">
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="H23" s="19"/>
+      <c r="H23" s="33"/>
       <c r="I23" s="10">
         <v>16</v>
       </c>
       <c r="J23" s="6">
         <v>46143</v>
       </c>
-      <c r="K23" s="4" t="s">
-        <v>60</v>
+      <c r="K23" s="4">
+        <v>46600</v>
       </c>
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
@@ -1679,15 +1772,27 @@
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
+      <c r="C24" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="H24" s="33"/>
+      <c r="I24" s="18">
+        <v>8</v>
+      </c>
+      <c r="J24" s="6">
+        <v>46174</v>
+      </c>
+      <c r="K24" s="4">
+        <v>46388</v>
+      </c>
       <c r="L24" s="16"/>
       <c r="M24" s="16"/>
       <c r="N24" s="16"/>
@@ -1699,15 +1804,27 @@
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
+      <c r="C25" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="H25" s="33"/>
+      <c r="I25" s="18">
+        <v>12</v>
+      </c>
+      <c r="J25" s="6">
+        <v>46174</v>
+      </c>
+      <c r="K25" s="4">
+        <v>46508</v>
+      </c>
       <c r="L25" s="16"/>
       <c r="M25" s="16"/>
       <c r="N25" s="16"/>
@@ -1719,17 +1836,27 @@
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
+      <c r="C26" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" s="33"/>
+      <c r="I26" s="30">
+        <v>4</v>
+      </c>
+      <c r="J26" s="6">
+        <v>46174</v>
+      </c>
+      <c r="K26" s="4">
+        <v>46266</v>
+      </c>
       <c r="L26" s="16"/>
       <c r="M26" s="16"/>
       <c r="N26" s="16"/>
@@ -1741,26 +1868,26 @@
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
-      <c r="C27" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="H27" s="19"/>
-      <c r="I27" s="10">
-        <v>6</v>
+      <c r="C27" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="33"/>
+      <c r="I27" s="30">
+        <v>16</v>
       </c>
       <c r="J27" s="6">
-        <v>45200</v>
+        <v>46174</v>
       </c>
       <c r="K27" s="4">
-        <v>45352</v>
+        <v>46631</v>
       </c>
       <c r="L27" s="16"/>
       <c r="M27" s="16"/>
@@ -1773,23 +1900,15 @@
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="2">
-        <v>45778</v>
-      </c>
-      <c r="K28" s="3">
-        <v>45992</v>
-      </c>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
       <c r="N28" s="16"/>
@@ -1801,15 +1920,17 @@
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" s="16"/>
       <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
+      <c r="C29" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="34"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="34"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="34"/>
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
       <c r="N29" s="16"/>
@@ -1821,15 +1942,27 @@
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="16"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
+      <c r="C30" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D30" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="H30" s="33"/>
+      <c r="I30" s="10">
+        <v>6</v>
+      </c>
+      <c r="J30" s="6">
+        <v>45200</v>
+      </c>
+      <c r="K30" s="4">
+        <v>45352</v>
+      </c>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
@@ -1841,15 +1974,23 @@
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" s="16"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
+      <c r="C31" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="31"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="2">
+        <v>45778</v>
+      </c>
+      <c r="K31" s="3">
+        <v>45992</v>
+      </c>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
       <c r="N31" s="16"/>
@@ -1959,6 +2100,7 @@
       <c r="R36" s="16"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A37" s="16"/>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
@@ -1977,8 +2119,67 @@
       <c r="Q37" s="16"/>
       <c r="R37" s="16"/>
     </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="16"/>
+      <c r="O38" s="16"/>
+      <c r="P38" s="16"/>
+      <c r="Q38" s="16"/>
+      <c r="R38" s="16"/>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="16"/>
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="Q39" s="16"/>
+      <c r="R39" s="16"/>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+    </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="44">
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D16:F16"/>
     <mergeCell ref="D17:F17"/>
@@ -2007,14 +2208,22 @@
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="G15:H15"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:H31"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="G20:H20"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="C29:K29"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="G26:H26"/>
     <mergeCell ref="D27:F27"/>
     <mergeCell ref="G27:H27"/>
-    <mergeCell ref="C26:K26"/>
-    <mergeCell ref="G22:H22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2033,46 +2242,52 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57DB3A5B-4E59-449D-BAB9-8505635379F5}">
-  <dimension ref="D8:S21"/>
+  <dimension ref="C8:S25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="1" max="1" width="2.21875" customWidth="1"/>
+    <col min="2" max="2" width="2" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" customWidth="1"/>
     <col min="4" max="4" width="24.77734375" customWidth="1"/>
     <col min="5" max="5" width="12.88671875" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="8" max="19" width="12.77734375" customWidth="1"/>
+    <col min="8" max="19" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D8" s="20" t="s">
+    <row r="8" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C8" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
-      <c r="Q8" s="20"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
-    </row>
-    <row r="9" spans="4:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="39"/>
+      <c r="S8" s="40"/>
+    </row>
+    <row r="9" spans="3:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="13" t="s">
+        <v>79</v>
+      </c>
       <c r="D9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
       <c r="H9" s="13" t="s">
         <v>46</v>
       </c>
@@ -2082,588 +2297,826 @@
       <c r="J9" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="K9" s="24" t="s">
+      <c r="K9" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="L9" s="24" t="s">
+      <c r="L9" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="M9" s="24" t="s">
+      <c r="M9" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="N9" s="24" t="s">
+      <c r="N9" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="O9" s="24" t="s">
+      <c r="O9" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="P9" s="24" t="s">
+      <c r="P9" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="Q9" s="24" t="s">
+      <c r="Q9" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="R9" s="24" t="s">
+      <c r="R9" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="S9" s="24" t="s">
+      <c r="S9" s="19" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="41" t="s">
+        <v>80</v>
+      </c>
       <c r="D10" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
       <c r="H10" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I10" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J10" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K10" s="14" t="s">
-        <v>59</v>
+        <v>67</v>
+      </c>
+      <c r="I10" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J10" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="21" t="s">
+        <v>67</v>
       </c>
       <c r="L10" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="N10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="O10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="P10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="S10" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S10" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="41" t="s">
+        <v>81</v>
+      </c>
       <c r="D11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
       <c r="H11" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J11" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="L11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="N11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="O11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="P11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R11" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="S11" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="I11" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J11" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="M11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S11" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="41" t="s">
+        <v>82</v>
+      </c>
       <c r="D12" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
       <c r="H12" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J12" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K12" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L12" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="M12" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="O12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="P12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="S12" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="I12" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J12" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K12" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="L12" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M12" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S12" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="41" t="s">
+        <v>83</v>
+      </c>
       <c r="D13" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
       <c r="H13" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J13" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K13" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L13" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="M13" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N13" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O13" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P13" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q13" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R13" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="S13" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="I13" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J13" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="L13" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M13" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N13" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O13" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P13" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q13" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R13" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S13" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="41" t="s">
+        <v>84</v>
+      </c>
       <c r="D14" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
       <c r="H14" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I14" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J14" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K14" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L14" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="M14" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N14" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O14" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P14" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q14" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R14" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="S14" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="I14" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J14" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K14" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="L14" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M14" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P14" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q14" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R14" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S14" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="41" t="s">
+        <v>85</v>
+      </c>
       <c r="D15" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
       <c r="H15" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I15" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J15" s="14" t="s">
-        <v>59</v>
+        <v>67</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J15" s="21" t="s">
+        <v>67</v>
       </c>
       <c r="K15" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="L15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="N15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="O15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="P15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="S15" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="M15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S15" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="41" t="s">
+        <v>86</v>
+      </c>
       <c r="D16" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
       <c r="H16" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="M16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="S16" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="I16" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J16" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M16" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N16" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O16" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P16" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q16" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R16" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S16" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="41" t="s">
+        <v>87</v>
+      </c>
       <c r="D17" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
       <c r="H17" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J17" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K17" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L17" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="M17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R17" s="26" t="s">
-        <v>58</v>
+        <v>67</v>
+      </c>
+      <c r="I17" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J17" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K17" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="L17" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M17" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N17" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O17" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P17" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q17" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R17" s="20" t="s">
+        <v>71</v>
       </c>
       <c r="S17" s="15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D18" s="14"/>
-      <c r="E18" s="19" t="s">
+    <row r="18" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="J18" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K18" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L18" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="M18" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N18" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O18" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P18" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q18" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R18" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="S18" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="19" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I18" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J18" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K18" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M18" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N18" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O18" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P18" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q18" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R18" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S18" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="41" t="s">
+        <v>89</v>
+      </c>
       <c r="D19" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="I19" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K19" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="L19" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="M19" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N19" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O19" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P19" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q19" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R19" s="15" t="s">
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L19" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M19" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N19" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O19" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P19" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q19" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R19" s="22" t="s">
         <v>31</v>
       </c>
       <c r="S19" s="15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="41" t="s">
+        <v>90</v>
+      </c>
       <c r="D20" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="J20" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K20" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="L20" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="M20" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N20" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O20" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P20" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q20" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R20" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="S20" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L20" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M20" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R20" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S20" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="41" t="s">
+        <v>91</v>
+      </c>
       <c r="D21" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K21" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="L21" s="14" t="s">
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L21" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="M21" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N21" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O21" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P21" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q21" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R21" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S21" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="41" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="M21" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="N21" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O21" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="P21" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q21" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="R21" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="S21" s="26" t="s">
-        <v>58</v>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="M22" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N22" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O22" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P22" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q22" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R22" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S22" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L23" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="M23" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S23" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C24" s="41" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="I24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="J24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="K24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M24" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N24" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O24" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P24" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="R24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="S24" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C25" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="I25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="J25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="K25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="L25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M25" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="N25" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O25" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="P25" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q25" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R25" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="S25" s="20" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="18">
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="C8:S8"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
     <mergeCell ref="E21:G21"/>
-    <mergeCell ref="D8:S8"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="E20:G20"/>
@@ -2678,21 +3131,32 @@
     <mergeCell ref="E10:G10"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H10:S21">
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="OK">
-      <formula>NOT(ISERROR(SEARCH("OK",H10)))</formula>
+  <conditionalFormatting sqref="H10:S25">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="NÃO INICIADO">
+      <formula>NOT(ISERROR(SEARCH("NÃO INICIADO",H10)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="!">
-      <formula>NOT(ISERROR(SEARCH("!",H10)))</formula>
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="EM PROGRESSO">
+      <formula>NOT(ISERROR(SEARCH("EM PROGRESSO",H10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="PENDENTE">
+      <formula>NOT(ISERROR(SEARCH("PENDENTE",H10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="ENVIADO">
+      <formula>NOT(ISERROR(SEARCH("ENVIADO",H10)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:S25" xr:uid="{C2B392FA-9EE8-4B53-B455-8FC23DA90C36}">
+      <formula1>status_name_list</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{C297617C-0740-451B-A447-4A6143CEBE6A}">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{31FF1D54-D4B0-4ADF-AA8B-44E61C543D9B}">
             <xm:f>NOT(ISERROR(SEARCH("-",H10)))</xm:f>
             <xm:f>"-"</xm:f>
             <x14:dxf>
@@ -2702,15 +3166,97 @@
               </font>
               <fill>
                 <patternFill>
-                  <bgColor theme="0" tint="-0.34998626667073579"/>
+                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
                 </patternFill>
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H10:S21</xm:sqref>
+          <xm:sqref>H10:S25</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC322B0-44FD-4547-9C83-0A2B861C218A}">
+  <dimension ref="B2:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="20.77734375" customWidth="1"/>
+    <col min="3" max="3" width="22.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B2" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="38"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B3" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B4" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B5" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B6" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B7" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B8" xr:uid="{22426952-A2F7-42CC-9255-59363FB29BE3}">
+      <formula1>status_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C8" xr:uid="{1608B37C-629C-4861-8DA4-ECE4BA0E272A}">
+      <formula1>status_name_list</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add and update some files in 'frequencias' folder
</commit_message>
<xml_diff>
--- a/arquivos/frequencias/apostilamento-frequencias.xlsx
+++ b/arquivos/frequencias/apostilamento-frequencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\arquivos\frequencias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E1B7DF-FF53-4B39-AB9F-D7CFE9D19546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC12A759-3470-4184-A21E-55EE7C7249CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8841256D-DED7-4986-96EA-3D864839F7ED}"/>
   </bookViews>
@@ -16,10 +16,13 @@
     <sheet name="MAIN" sheetId="1" r:id="rId1"/>
     <sheet name="2025" sheetId="3" r:id="rId2"/>
     <sheet name="2026" sheetId="2" r:id="rId3"/>
-    <sheet name="CONFIG" sheetId="4" r:id="rId4"/>
+    <sheet name="2027" sheetId="6" r:id="rId4"/>
+    <sheet name="CONFIG" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="status_list" localSheetId="3">tbl_status[status_id]</definedName>
     <definedName name="status_list">tbl_status[status_id]</definedName>
+    <definedName name="status_name_list" localSheetId="3">tbl_status[display_name]</definedName>
     <definedName name="status_name_list">tbl_status[display_name]</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -44,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="100">
   <si>
     <t>APENADO</t>
   </si>
@@ -181,9 +184,6 @@
     <t>9000011-71.2025.8.15.0561</t>
   </si>
   <si>
-    <t>FREQUÊNCIAS</t>
-  </si>
-  <si>
     <t>JANEIRO</t>
   </si>
   <si>
@@ -332,6 +332,21 @@
   </si>
   <si>
     <t>AF0016</t>
+  </si>
+  <si>
+    <t>FREQUÊNCIAS  2026</t>
+  </si>
+  <si>
+    <t>FREQUÊNCIAS  2027</t>
+  </si>
+  <si>
+    <t>AF0017</t>
+  </si>
+  <si>
+    <t>TAYSE APOLIANA CARMO</t>
+  </si>
+  <si>
+    <t>JOSÉ SILDO GREGÓRIO</t>
   </si>
 </sst>
 </file>
@@ -545,7 +560,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -619,10 +634,26 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -636,76 +667,20 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="21">
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -800,6 +775,171 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -814,14 +954,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67B21386-A7FE-4230-BF7C-AC6702050BBE}" name="tbl_status" displayName="tbl_status" ref="B3:C8" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67B21386-A7FE-4230-BF7C-AC6702050BBE}" name="tbl_status" displayName="tbl_status" ref="B3:C8" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="B3:C8" xr:uid="{67B21386-A7FE-4230-BF7C-AC6702050BBE}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{8CA856E5-CBA8-4981-BAC5-458B8D165D4E}" name="status_id" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{DEF6E58C-573F-4688-813D-EB15040558D7}" name="display_name" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{8CA856E5-CBA8-4981-BAC5-458B8D165D4E}" name="status_id" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{DEF6E58C-573F-4688-813D-EB15040558D7}" name="display_name" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1124,7 +1264,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EF9E8C-546D-4B9E-9D3D-4B096DC9D66B}">
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="28.21875" customWidth="1"/>
@@ -1282,17 +1422,17 @@
     <row r="8" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="40"/>
+      <c r="K8" s="40"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
@@ -1307,15 +1447,15 @@
       <c r="C9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="36" t="s">
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="36"/>
+      <c r="H9" s="42"/>
       <c r="I9" s="8" t="s">
         <v>30</v>
       </c>
@@ -1339,15 +1479,15 @@
       <c r="C10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31" t="s">
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="31"/>
+      <c r="H10" s="38"/>
       <c r="I10" s="7">
         <v>7</v>
       </c>
@@ -1371,15 +1511,15 @@
       <c r="C11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="31" t="s">
+      <c r="D11" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="32" t="s">
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="H11" s="32"/>
+      <c r="H11" s="39"/>
       <c r="I11" s="9">
         <v>8</v>
       </c>
@@ -1403,15 +1543,15 @@
       <c r="C12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="32" t="s">
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="32"/>
+      <c r="H12" s="39"/>
       <c r="I12" s="9">
         <v>8</v>
       </c>
@@ -1435,15 +1575,15 @@
       <c r="C13" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="D13" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="32" t="s">
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="32"/>
+      <c r="H13" s="39"/>
       <c r="I13" s="9">
         <v>4</v>
       </c>
@@ -1467,15 +1607,15 @@
       <c r="C14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="32" t="s">
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="32"/>
+      <c r="H14" s="39"/>
       <c r="I14" s="9">
         <v>14</v>
       </c>
@@ -1499,15 +1639,15 @@
       <c r="C15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="32" t="s">
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="32"/>
+      <c r="H15" s="39"/>
       <c r="I15" s="9">
         <v>12</v>
       </c>
@@ -1531,15 +1671,15 @@
       <c r="C16" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="32" t="s">
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="H16" s="32"/>
+      <c r="H16" s="39"/>
       <c r="I16" s="9">
         <v>12</v>
       </c>
@@ -1563,15 +1703,15 @@
       <c r="C17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="D17" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="H17" s="32"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" s="39"/>
       <c r="I17" s="9" t="s">
         <v>31</v>
       </c>
@@ -1591,15 +1731,15 @@
       <c r="C18" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="32"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="H18" s="39"/>
       <c r="I18" s="9" t="s">
         <v>31</v>
       </c>
@@ -1621,15 +1761,15 @@
       <c r="C19" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="31" t="s">
+      <c r="D19" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" s="32"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" s="39"/>
       <c r="I19" s="9" t="s">
         <v>31</v>
       </c>
@@ -1647,15 +1787,15 @@
       <c r="A20" s="16"/>
       <c r="B20" s="16"/>
       <c r="C20" s="7"/>
-      <c r="D20" s="33" t="s">
+      <c r="D20" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33" t="s">
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="33"/>
+      <c r="H20" s="37"/>
       <c r="I20" s="10">
         <v>12</v>
       </c>
@@ -1679,15 +1819,15 @@
       <c r="C21" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="33" t="s">
+      <c r="D21" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33" t="s">
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="H21" s="33"/>
+      <c r="H21" s="37"/>
       <c r="I21" s="10">
         <v>5</v>
       </c>
@@ -1711,15 +1851,15 @@
       <c r="C22" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33" t="s">
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="H22" s="33"/>
+      <c r="H22" s="37"/>
       <c r="I22" s="10">
         <v>24</v>
       </c>
@@ -1743,15 +1883,15 @@
       <c r="C23" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33" t="s">
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="H23" s="33"/>
+      <c r="H23" s="37"/>
       <c r="I23" s="10">
         <v>16</v>
       </c>
@@ -1773,17 +1913,17 @@
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
       <c r="C24" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33" t="s">
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="H24" s="33"/>
+      <c r="H24" s="37"/>
       <c r="I24" s="18">
         <v>8</v>
       </c>
@@ -1805,17 +1945,17 @@
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
       <c r="C25" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="H25" s="33"/>
+      <c r="D25" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H25" s="37"/>
       <c r="I25" s="18">
         <v>12</v>
       </c>
@@ -1837,17 +1977,17 @@
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
       <c r="C26" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="D26" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="D26" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33" t="s">
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="H26" s="33"/>
+      <c r="H26" s="37"/>
       <c r="I26" s="30">
         <v>4</v>
       </c>
@@ -1869,17 +2009,17 @@
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
       <c r="C27" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="D27" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33" t="s">
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="H27" s="33"/>
+      <c r="H27" s="37"/>
       <c r="I27" s="30">
         <v>16</v>
       </c>
@@ -1900,15 +2040,27 @@
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
+      <c r="C28" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" s="37"/>
+      <c r="I28" s="36">
+        <v>4</v>
+      </c>
+      <c r="J28" s="6">
+        <v>46204</v>
+      </c>
+      <c r="K28" s="4">
+        <v>46296</v>
+      </c>
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
       <c r="N28" s="16"/>
@@ -1920,17 +2072,15 @@
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" s="16"/>
       <c r="B29" s="16"/>
-      <c r="C29" s="34" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
       <c r="N29" s="16"/>
@@ -1942,27 +2092,17 @@
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="16"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D30" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="H30" s="33"/>
-      <c r="I30" s="10">
-        <v>6</v>
-      </c>
-      <c r="J30" s="6">
-        <v>45200</v>
-      </c>
-      <c r="K30" s="4">
-        <v>45352</v>
-      </c>
+      <c r="C30" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="40"/>
+      <c r="J30" s="40"/>
+      <c r="K30" s="40"/>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
@@ -1974,22 +2114,26 @@
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" s="16"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" s="31" t="s">
-        <v>5</v>
-      </c>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="2">
-        <v>45778</v>
-      </c>
-      <c r="K31" s="3">
-        <v>45992</v>
+      <c r="C31" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D31" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="H31" s="37"/>
+      <c r="I31" s="10">
+        <v>6</v>
+      </c>
+      <c r="J31" s="6">
+        <v>45200</v>
+      </c>
+      <c r="K31" s="4">
+        <v>45352</v>
       </c>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
@@ -2002,15 +2146,23 @@
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" s="16"/>
       <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16"/>
+      <c r="C32" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="38" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="2">
+        <v>45778</v>
+      </c>
+      <c r="K32" s="3">
+        <v>45992</v>
+      </c>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
       <c r="N32" s="16"/>
@@ -2160,6 +2312,7 @@
       <c r="R39" s="16"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A40" s="16"/>
       <c r="B40" s="16"/>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
@@ -2178,20 +2331,43 @@
       <c r="Q40" s="16"/>
       <c r="R40" s="16"/>
     </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="16"/>
+      <c r="G41" s="16"/>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="16"/>
+      <c r="L41" s="16"/>
+      <c r="M41" s="16"/>
+      <c r="N41" s="16"/>
+      <c r="O41" s="16"/>
+      <c r="P41" s="16"/>
+      <c r="Q41" s="16"/>
+      <c r="R41" s="16"/>
+    </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="D18:F18"/>
+  <mergeCells count="46">
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="C30:K30"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="G27:H27"/>
     <mergeCell ref="C8:K8"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="G23:H23"/>
@@ -2208,22 +2384,20 @@
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="G15:H15"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="C29:K29"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="D18:F18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2242,6 +2416,1077 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57DB3A5B-4E59-449D-BAB9-8505635379F5}">
+  <dimension ref="C8:S27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.21875" customWidth="1"/>
+    <col min="2" max="2" width="2" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="24.77734375" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="19" width="15.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C8" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="44"/>
+      <c r="O8" s="44"/>
+      <c r="P8" s="44"/>
+      <c r="Q8" s="44"/>
+      <c r="R8" s="44"/>
+      <c r="S8" s="45"/>
+    </row>
+    <row r="9" spans="3:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="L9" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="M9" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="N9" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="O9" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="P9" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q9" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="R9" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="S9" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J10" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K10" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="M10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R10" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S10" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="M11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S11" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J12" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K12" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L12" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M12" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S12" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J13" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K13" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L13" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M13" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N13" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O13" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P13" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q13" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R13" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S13" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J14" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K14" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L14" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S14" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J15" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K15" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="L15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="M15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="O15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="P15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S15" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J16" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K16" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L16" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N16" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S16" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="J17" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="K17" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L17" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M17" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N17" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O17" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P17" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q17" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R17" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S17" s="15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I18" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J18" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K18" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M18" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N18" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S18" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L19" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N19" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O19" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P19" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q19" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="R19" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="S19" s="15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K20" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L20" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M20" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N20" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S20" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K21" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L21" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M21" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N21" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S21" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="M22" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N22" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O22" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P22" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q22" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R22" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S22" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L23" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="M23" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N23" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S23" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C24" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="I24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="J24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="K24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M24" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N24" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O24" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P24" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="R24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="S24" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C25" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="I25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="J25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="K25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="L25" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M25" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N25" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S25" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C26" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="I26" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="J26" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="K26" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="L26" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="M26" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="N26" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O26" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P26" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q26" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R26" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="S26" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C27" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="I27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="J27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="K27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="L27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="M27" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="N27" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O27" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P27" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q27" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="R27" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="S27" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="C8:S8"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E25:G25"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="H10:S26">
+    <cfRule type="containsText" dxfId="20" priority="6" operator="containsText" text="NÃO INICIADO">
+      <formula>NOT(ISERROR(SEARCH("NÃO INICIADO",H10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="19" priority="7" operator="containsText" text="EM PROGRESSO">
+      <formula>NOT(ISERROR(SEARCH("EM PROGRESSO",H10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="8" operator="containsText" text="PENDENTE">
+      <formula>NOT(ISERROR(SEARCH("PENDENTE",H10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="17" priority="10" operator="containsText" text="ENVIADO">
+      <formula>NOT(ISERROR(SEARCH("ENVIADO",H10)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27:S27">
+    <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="NÃO INICIADO">
+      <formula>NOT(ISERROR(SEARCH("NÃO INICIADO",H27)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="EM PROGRESSO">
+      <formula>NOT(ISERROR(SEARCH("EM PROGRESSO",H27)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="PENDENTE">
+      <formula>NOT(ISERROR(SEARCH("PENDENTE",H27)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="13" priority="5" operator="containsText" text="ENVIADO">
+      <formula>NOT(ISERROR(SEARCH("ENVIADO",H27)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:S27" xr:uid="{C2B392FA-9EE8-4B53-B455-8FC23DA90C36}">
+      <formula1>status_name_list</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="9" operator="containsText" id="{31FF1D54-D4B0-4ADF-AA8B-44E61C543D9B}">
+            <xm:f>NOT(ISERROR(SEARCH("-",H10)))</xm:f>
+            <xm:f>"-"</xm:f>
+            <x14:dxf>
+              <font>
+                <b/>
+                <i val="0"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>H10:S26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{13FF8B9E-8E68-47E2-8866-313BDFA1A65D}">
+            <xm:f>NOT(ISERROR(SEARCH("-",H27)))</xm:f>
+            <xm:f>"-"</xm:f>
+            <x14:dxf>
+              <font>
+                <b/>
+                <i val="0"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>H27:S27</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B133746-E17F-40AF-9BB2-98ACABC5DBCD}">
   <dimension ref="C8:S25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2256,897 +3501,896 @@
   </cols>
   <sheetData>
     <row r="8" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C8" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="39"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="39"/>
-      <c r="L8" s="39"/>
-      <c r="M8" s="39"/>
-      <c r="N8" s="39"/>
-      <c r="O8" s="39"/>
-      <c r="P8" s="39"/>
-      <c r="Q8" s="39"/>
-      <c r="R8" s="39"/>
-      <c r="S8" s="40"/>
+      <c r="C8" s="44" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="44"/>
+      <c r="O8" s="44"/>
+      <c r="P8" s="44"/>
+      <c r="Q8" s="44"/>
+      <c r="R8" s="44"/>
+      <c r="S8" s="45"/>
     </row>
     <row r="9" spans="3:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
       <c r="H9" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="K9" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="K9" s="19" t="s">
+      <c r="L9" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="M9" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="M9" s="19" t="s">
+      <c r="N9" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="O9" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="O9" s="19" t="s">
+      <c r="P9" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="P9" s="19" t="s">
+      <c r="Q9" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="Q9" s="19" t="s">
+      <c r="R9" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="R9" s="19" t="s">
+      <c r="S9" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="S9" s="19" t="s">
+    </row>
+    <row r="10" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R10" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S10" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S11" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R12" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S12" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R13" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S13" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="M14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R14" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S14" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R15" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S15" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="M16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="O16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R16" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S16" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R17" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S17" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S18" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="I19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="J19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="L19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="M19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="O19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="P19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S19" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="M20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="O20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="S20" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="M21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="O21" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P21" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q21" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="R21" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="S21" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" s="31" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C10" s="41" t="s">
-        <v>80</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I10" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J10" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K10" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="M10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="N10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="O10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="P10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="R10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="S10" s="22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="31" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I11" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J11" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="L11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="M11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="N11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="O11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="P11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="R11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="S11" s="22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="41" t="s">
-        <v>82</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="31" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" s="31"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I12" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J12" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K12" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L12" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M12" s="20" t="s">
+      <c r="E22" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="J22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="K22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="M22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="N22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="O22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="P22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="R22" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="S22" s="31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="N12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="O12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="P12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="R12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="S12" s="22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="31" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I13" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J13" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K13" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L13" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M13" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N13" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O13" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P13" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q13" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R13" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S13" s="22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="41" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I14" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J14" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K14" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L14" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M14" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N14" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O14" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P14" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q14" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R14" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S14" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="41" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I15" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J15" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K15" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="L15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="M15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="N15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="O15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="P15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="R15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="S15" s="22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="41" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I16" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J16" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K16" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L16" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M16" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N16" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O16" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P16" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q16" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R16" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S16" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="41" t="s">
-        <v>87</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="I17" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="J17" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="K17" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L17" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M17" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N17" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O17" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P17" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q17" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R17" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S17" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="41" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I18" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="J18" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K18" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="L18" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M18" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N18" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O18" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P18" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q18" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R18" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S18" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="19" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="41" t="s">
-        <v>89</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I19" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="J19" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K19" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="L19" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M19" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N19" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O19" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P19" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q19" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="R19" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="S19" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="20" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="41" t="s">
-        <v>90</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E20" s="33" t="s">
-        <v>37</v>
-      </c>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I20" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="J20" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K20" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="L20" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M20" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N20" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O20" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P20" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q20" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R20" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S20" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="21" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="41" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="E21" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I21" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="J21" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K21" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="L21" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M21" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N21" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O21" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P21" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q21" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R21" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S21" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="22" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="41" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="E22" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I22" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="J22" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K22" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="L22" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="M22" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N22" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O22" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P22" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q22" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R22" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S22" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="41" t="s">
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L23" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="M23" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="N23" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="O23" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="P23" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q23" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="R23" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="S23" s="31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C24" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="E23" s="33" t="s">
+      <c r="D24" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I23" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="J23" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K23" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="L23" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="M23" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N23" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O23" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P23" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q23" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="R23" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="S23" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C24" s="41" t="s">
+      <c r="E24" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="I24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="J24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="M24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="N24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="O24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="P24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="R24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="S24" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="C25" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="33" t="s">
+      <c r="D25" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="I24" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="J24" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="K24" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="L24" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="M24" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="N24" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O24" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P24" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q24" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="R24" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="S24" s="20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="25" spans="3:19" x14ac:dyDescent="0.3">
-      <c r="C25" s="41" t="s">
-        <v>95</v>
-      </c>
-      <c r="D25" s="29" t="s">
+      <c r="E25" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="I25" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="J25" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="K25" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="L25" s="29" t="s">
-        <v>31</v>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="I25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="K25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L25" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="M25" s="20" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N25" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O25" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P25" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q25" s="20" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="R25" s="20" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="S25" s="20" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="E24:G24"/>
     <mergeCell ref="E25:G25"/>
-    <mergeCell ref="C8:S8"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E17:G17"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="E24:G24"/>
     <mergeCell ref="E13:G13"/>
-    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="C8:S8"/>
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E12:G12"/>
   </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="H10:S25">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="NÃO INICIADO">
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="NÃO INICIADO">
       <formula>NOT(ISERROR(SEARCH("NÃO INICIADO",H10)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="EM PROGRESSO">
+    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="EM PROGRESSO">
       <formula>NOT(ISERROR(SEARCH("EM PROGRESSO",H10)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="PENDENTE">
+    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="PENDENTE">
       <formula>NOT(ISERROR(SEARCH("PENDENTE",H10)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="ENVIADO">
+    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="ENVIADO">
       <formula>NOT(ISERROR(SEARCH("ENVIADO",H10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:S25" xr:uid="{C2B392FA-9EE8-4B53-B455-8FC23DA90C36}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:S25" xr:uid="{E39F1B19-1BDE-4288-8C74-7A6265CD120C}">
       <formula1>status_name_list</formula1>
     </dataValidation>
   </dataValidations>
@@ -3156,7 +4400,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{31FF1D54-D4B0-4ADF-AA8B-44E61C543D9B}">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{8F7D0E32-63CA-4BBD-9B70-A5A53A1D1647}">
             <xm:f>NOT(ISERROR(SEARCH("-",H10)))</xm:f>
             <xm:f>"-"</xm:f>
             <x14:dxf>
@@ -3179,7 +4423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC322B0-44FD-4547-9C83-0A2B861C218A}">
   <dimension ref="B2:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3189,54 +4433,54 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" s="38"/>
+      <c r="B2" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="46"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="28" t="s">
         <v>63</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>31</v>

</xml_diff>